<commit_message>
docs: nome da clinica na planilha e metadados dos documentos gerados
A planilha de custos passa a trazer "Jaqueline Aranha Estetica" no titulo e nas propriedades
do arquivo, e sai sem o caminho da pasta local que o Excel grava ao salvar. Os DOCX/PDF
gerados ganham titulo, assunto e autor nas propriedades (antes: autor "python-docx").

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tcc/JaquelineAranhaEstetica-Custos-Operacionais.xlsx
+++ b/docs/tcc/JaquelineAranhaEstetica-Custos-Operacionais.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafae\Documents\shivazen-app\docs\tcc\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3819EB02-E0E1-4053-8073-A76F469A2C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6035B72F-2B68-41CF-AAC3-E86BA9FDD3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +31,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="125">
   <si>
-    <t>Custo do sistema: clínica com até 60 atendimentos por mês</t>
+    <t>Jaqueline Aranha Estética: custo do sistema para até 60 atendimentos por mês</t>
   </si>
   <si>
     <t>Células em azul são entradas: troque o valor e a planilha recalcula. Preços de lista consultados em 30/10/2026; endereços na aba Fontes.</t>

</xml_diff>